<commit_message>
fix: removed counting of false api calls.
</commit_message>
<xml_diff>
--- a/experiment/meta-llama-llama-4-scout-17b-16e-instruct_Experiment.xlsx
+++ b/experiment/meta-llama-llama-4-scout-17b-16e-instruct_Experiment.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -543,7 +543,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>3984</v>
+        <v>3540</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -553,21 +553,84 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>1535</v>
+        <v>1257</v>
       </c>
       <c r="O2" t="n">
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>0.0005219000000000001</v>
+        <v>0.00042738</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>0.0009601400000000001</v>
+        <v>0.00081678</v>
       </c>
       <c r="S2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>grade school math problems</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-4-scout-17b-16e-instruct</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>12</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>(1.0, 1.0)</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>2463</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>965</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.0003281</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.00059903</v>
+      </c>
+      <c r="S3" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Experiments now test mmlu.
</commit_message>
<xml_diff>
--- a/experiment/meta-llama-llama-4-scout-17b-16e-instruct_Experiment.xlsx
+++ b/experiment/meta-llama-llama-4-scout-17b-16e-instruct_Experiment.xlsx
@@ -413,105 +413,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>agents</t>
+          <t>basic math problems</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>rounds</t>
+          <t>grade school math problems</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>eval_rounds</t>
+          <t>biography problems</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>model</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>api_calls</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>accuracy</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>standard error</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>confidence interval</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>input_tokens_used</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>input_tokens_saved</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>input_ cost ($)</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>input_cost_saved ($)</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>output_tokens_used</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>output_tokens_saved</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>output_cost ($)</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>output_cost_saved ($)</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>cost ($)</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>cost_saved ($)</t>
+          <t>mmlu problems</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>basic math problems</t>
+          <t>agents</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -521,60 +451,16 @@
         <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>meta-llama/llama-4-scout-17b-16e-instruct</t>
-        </is>
-      </c>
-      <c r="F2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>(1.0, 1.0)</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>3540</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="n">
-        <v>1257</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.00042738</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0.00081678</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
+        <v>3</v>
+      </c>
+      <c r="E2" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>grade school math problems</t>
+          <t>rounds</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -584,54 +470,322 @@
         <v>2</v>
       </c>
       <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>eval_rounds</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>meta-llama/llama-4-scout-17b-16e-instruct</t>
         </is>
       </c>
-      <c r="F3" t="n">
-        <v>12</v>
-      </c>
-      <c r="G3" t="n">
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-4-scout-17b-16e-instruct</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-4-scout-17b-16e-instruct</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-4-scout-17b-16e-instruct</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>api_calls</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>accuracy</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>1</v>
       </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="inlineStr">
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>standard error</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.1521200048243774</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>confidence interval</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>(1.0, 1.0)</t>
         </is>
       </c>
-      <c r="J3" t="n">
-        <v>2463</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" t="n">
-        <v>965</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0.0003281</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0.00059903</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0</v>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>(1.0, 1.0)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>(0.024691870722828912, 0.7025808565498983)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>(1.0, 1.0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>input_tokens_used</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3230</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2391</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>input_tokens_saved</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3366</v>
+      </c>
+      <c r="E11" t="n">
+        <v>5304</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>input_ cost ($)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>input_cost_saved ($)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.00037026</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.0005834400000000001</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>output_tokens_used</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1087</v>
+      </c>
+      <c r="C14" t="n">
+        <v>919</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>output_tokens_saved</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>2275</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2817</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>output_cost ($)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.00036958</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.00031246</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>output_cost_saved ($)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.0007735</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.0009577800000000001</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>cost ($)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.00072488</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.00057547</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>cost_saved ($)</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.00114376</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0.00154122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: change the names of importet inference clients, so they are not accidentally.
</commit_message>
<xml_diff>
--- a/experiment/meta-llama-llama-4-scout-17b-16e-instruct_Experiment.xlsx
+++ b/experiment/meta-llama-llama-4-scout-17b-16e-instruct_Experiment.xlsx
@@ -554,7 +554,7 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>0.36</v>
+        <v>0.33</v>
       </c>
       <c r="E7" t="n">
         <v>1</v>
@@ -573,7 +573,7 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1521200048243774</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -597,7 +597,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>(0.024691870722828912, 0.7025808565498983)</t>
+          <t>(-0.05100068920069428, 0.717667355867361)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -613,10 +613,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3230</v>
+        <v>3682</v>
       </c>
       <c r="C10" t="n">
-        <v>2391</v>
+        <v>2040</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
@@ -638,22 +638,30 @@
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>3366</v>
+        <v>2919</v>
       </c>
       <c r="E11" t="n">
-        <v>5304</v>
+        <v>4809</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>input_ cost ($)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
+          <t>input_cost ($)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.00040502</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.0002244</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -668,10 +676,10 @@
         <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>0.00037026</v>
+        <v>0.0003210899999999999</v>
       </c>
       <c r="E13" t="n">
-        <v>0.0005834400000000001</v>
+        <v>0.00052899</v>
       </c>
     </row>
     <row r="14">
@@ -681,10 +689,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1087</v>
+        <v>1351</v>
       </c>
       <c r="C14" t="n">
-        <v>919</v>
+        <v>799</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -706,10 +714,10 @@
         <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>2275</v>
+        <v>2216</v>
       </c>
       <c r="E15" t="n">
-        <v>2817</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="16">
@@ -719,10 +727,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.00036958</v>
+        <v>0.00045934</v>
       </c>
       <c r="C16" t="n">
-        <v>0.00031246</v>
+        <v>0.00027166</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
@@ -744,10 +752,10 @@
         <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0007735</v>
+        <v>0.0007534400000000001</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0009577800000000001</v>
+        <v>0.0008377600000000001</v>
       </c>
     </row>
     <row r="18">
@@ -757,10 +765,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.00072488</v>
+        <v>0.00086436</v>
       </c>
       <c r="C18" t="n">
-        <v>0.00057547</v>
+        <v>0.00049606</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -782,10 +790,10 @@
         <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>0.00114376</v>
+        <v>0.00107453</v>
       </c>
       <c r="E19" t="n">
-        <v>0.00154122</v>
+        <v>0.00136675</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: fixed wrong handling of metadata.
</commit_message>
<xml_diff>
--- a/experiment/meta-llama-llama-4-scout-17b-16e-instruct_Experiment.xlsx
+++ b/experiment/meta-llama-llama-4-scout-17b-16e-instruct_Experiment.xlsx
@@ -413,28 +413,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>basic math problems</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>grade school math problems</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
           <t>biography problems</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>mmlu problems</t>
         </is>
       </c>
     </row>
@@ -445,15 +430,6 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -464,15 +440,6 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E3" t="n">
         <v>2</v>
       </c>
     </row>
@@ -485,15 +452,6 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -506,21 +464,6 @@
           <t>meta-llama/llama-4-scout-17b-16e-instruct</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>meta-llama/llama-4-scout-17b-16e-instruct</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>meta-llama/llama-4-scout-17b-16e-instruct</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>meta-llama/llama-4-scout-17b-16e-instruct</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -531,15 +474,6 @@
       <c r="B6" t="n">
         <v>6</v>
       </c>
-      <c r="C6" t="n">
-        <v>6</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
-        <v>6</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -548,16 +482,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="E7" t="n">
-        <v>1</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -567,16 +492,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0.1666666666666667</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
+        <v>0.1756820922315766</v>
       </c>
     </row>
     <row r="9">
@@ -587,22 +503,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>(1.0, 1.0)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>(1.0, 1.0)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>(-0.05100068920069428, 0.717667355867361)</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>(1.0, 1.0)</t>
+          <t>(0.15043192438822023, 0.960679186722891)</t>
         </is>
       </c>
     </row>
@@ -613,16 +514,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3682</v>
-      </c>
-      <c r="C10" t="n">
-        <v>2040</v>
-      </c>
-      <c r="D10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
+        <v>3267</v>
       </c>
     </row>
     <row r="11">
@@ -634,15 +526,6 @@
       <c r="B11" t="n">
         <v>0</v>
       </c>
-      <c r="C11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" t="n">
-        <v>2919</v>
-      </c>
-      <c r="E11" t="n">
-        <v>4809</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -651,16 +534,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.00040502</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0.0002244</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0</v>
+        <v>0.00035937</v>
       </c>
     </row>
     <row r="13">
@@ -672,15 +546,6 @@
       <c r="B13" t="n">
         <v>0</v>
       </c>
-      <c r="C13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0.0003210899999999999</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0.00052899</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -689,16 +554,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1351</v>
-      </c>
-      <c r="C14" t="n">
-        <v>799</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0</v>
+        <v>2291</v>
       </c>
     </row>
     <row r="15">
@@ -710,15 +566,6 @@
       <c r="B15" t="n">
         <v>0</v>
       </c>
-      <c r="C15" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" t="n">
-        <v>2216</v>
-      </c>
-      <c r="E15" t="n">
-        <v>2464</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -727,16 +574,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.00045934</v>
-      </c>
-      <c r="C16" t="n">
-        <v>0.00027166</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0</v>
+        <v>0.0007789400000000001</v>
       </c>
     </row>
     <row r="17">
@@ -748,15 +586,6 @@
       <c r="B17" t="n">
         <v>0</v>
       </c>
-      <c r="C17" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0.0007534400000000001</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0.0008377600000000001</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -765,16 +594,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.00086436</v>
-      </c>
-      <c r="C18" t="n">
-        <v>0.00049606</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0</v>
+        <v>0.00113831</v>
       </c>
     </row>
     <row r="19">
@@ -785,15 +605,6 @@
       </c>
       <c r="B19" t="n">
         <v>0</v>
-      </c>
-      <c r="C19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0.00107453</v>
-      </c>
-      <c r="E19" t="n">
-        <v>0.00136675</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: moved now all calculation of cost out from gen_.
</commit_message>
<xml_diff>
--- a/experiment/meta-llama-llama-4-scout-17b-16e-instruct_Experiment.xlsx
+++ b/experiment/meta-llama-llama-4-scout-17b-16e-instruct_Experiment.xlsx
@@ -413,13 +413,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
+          <t>basic math problems</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>grade school math problems</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>biography problems</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>mmlu problems</t>
         </is>
       </c>
     </row>
@@ -430,6 +445,15 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -440,6 +464,15 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
         <v>2</v>
       </c>
     </row>
@@ -452,6 +485,15 @@
       <c r="B4" t="n">
         <v>1</v>
       </c>
+      <c r="C4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -464,6 +506,21 @@
           <t>meta-llama/llama-4-scout-17b-16e-instruct</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-4-scout-17b-16e-instruct</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-4-scout-17b-16e-instruct</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>meta-llama/llama-4-scout-17b-16e-instruct</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -474,6 +531,15 @@
       <c r="B6" t="n">
         <v>6</v>
       </c>
+      <c r="C6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -482,7 +548,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.5600000000000001</v>
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -492,7 +567,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.1756820922315766</v>
+        <v>0</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.1521200048243774</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -503,7 +587,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>(0.15043192438822023, 0.960679186722891)</t>
+          <t>(1.0, 1.0)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>(1.0, 1.0)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>(0.2974191434501016, 0.975308129277171)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>(1.0, 1.0)</t>
         </is>
       </c>
     </row>
@@ -514,7 +613,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3267</v>
+        <v>3492</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2442</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3591</v>
+      </c>
+      <c r="E10" t="n">
+        <v>5187</v>
       </c>
     </row>
     <row r="11">
@@ -526,6 +634,15 @@
       <c r="B11" t="n">
         <v>0</v>
       </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -534,7 +651,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.00035937</v>
+        <v>0.00038412</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.00026862</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.00039501</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.0005705700000000001</v>
       </c>
     </row>
     <row r="13">
@@ -546,6 +672,15 @@
       <c r="B13" t="n">
         <v>0</v>
       </c>
+      <c r="C13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -554,7 +689,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2291</v>
+        <v>1320</v>
+      </c>
+      <c r="C14" t="n">
+        <v>961</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2438</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2674</v>
       </c>
     </row>
     <row r="15">
@@ -566,6 +710,15 @@
       <c r="B15" t="n">
         <v>0</v>
       </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -574,7 +727,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.0007789400000000001</v>
+        <v>0.0004488</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.00032674</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.00082892</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.0009091600000000001</v>
       </c>
     </row>
     <row r="17">
@@ -586,6 +748,15 @@
       <c r="B17" t="n">
         <v>0</v>
       </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -594,7 +765,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.00113831</v>
+        <v>0.00083292</v>
+      </c>
+      <c r="C18" t="n">
+        <v>0.0005953600000000001</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0.00122393</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0.00147973</v>
       </c>
     </row>
     <row r="19">
@@ -604,6 +784,15 @@
         </is>
       </c>
       <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: now also counts tokens used eval_convesation.py.
</commit_message>
<xml_diff>
--- a/experiment/meta-llama-llama-4-scout-17b-16e-instruct_Experiment.xlsx
+++ b/experiment/meta-llama-llama-4-scout-17b-16e-instruct_Experiment.xlsx
@@ -535,10 +535,10 @@
         <v>6</v>
       </c>
       <c r="D6" t="n">
+        <v>27</v>
+      </c>
+      <c r="E6" t="n">
         <v>6</v>
-      </c>
-      <c r="E6" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="7">
@@ -554,7 +554,7 @@
         <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>0.64</v>
+        <v>0.55</v>
       </c>
       <c r="E7" t="n">
         <v>1</v>
@@ -573,7 +573,7 @@
         <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1521200048243774</v>
+        <v>0.1574591643244434</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
@@ -597,7 +597,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>(0.2974191434501016, 0.975308129277171)</t>
+          <t>(0.194613663821962, 0.8962954270871288)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -613,16 +613,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3492</v>
+        <v>3262</v>
       </c>
       <c r="C10" t="n">
-        <v>2442</v>
+        <v>2370</v>
       </c>
       <c r="D10" t="n">
-        <v>3591</v>
+        <v>13613</v>
       </c>
       <c r="E10" t="n">
-        <v>5187</v>
+        <v>5238</v>
       </c>
     </row>
     <row r="11">
@@ -651,16 +651,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.00038412</v>
+        <v>0.00035882</v>
       </c>
       <c r="C12" t="n">
-        <v>0.00026862</v>
+        <v>0.0002607</v>
       </c>
       <c r="D12" t="n">
-        <v>0.00039501</v>
+        <v>0.00149743</v>
       </c>
       <c r="E12" t="n">
-        <v>0.0005705700000000001</v>
+        <v>0.0005761799999999999</v>
       </c>
     </row>
     <row r="13">
@@ -689,16 +689,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1320</v>
+        <v>1228</v>
       </c>
       <c r="C14" t="n">
-        <v>961</v>
+        <v>944</v>
       </c>
       <c r="D14" t="n">
-        <v>2438</v>
+        <v>3490</v>
       </c>
       <c r="E14" t="n">
-        <v>2674</v>
+        <v>2403</v>
       </c>
     </row>
     <row r="15">
@@ -727,16 +727,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.0004488</v>
+        <v>0.0004175200000000001</v>
       </c>
       <c r="C16" t="n">
-        <v>0.00032674</v>
+        <v>0.00032096</v>
       </c>
       <c r="D16" t="n">
-        <v>0.00082892</v>
+        <v>0.0011866</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0009091600000000001</v>
+        <v>0.0008170200000000001</v>
       </c>
     </row>
     <row r="17">
@@ -765,16 +765,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.00083292</v>
+        <v>0.00077634</v>
       </c>
       <c r="C18" t="n">
-        <v>0.0005953600000000001</v>
+        <v>0.00058166</v>
       </c>
       <c r="D18" t="n">
-        <v>0.00122393</v>
+        <v>0.00268403</v>
       </c>
       <c r="E18" t="n">
-        <v>0.00147973</v>
+        <v>0.0013932</v>
       </c>
     </row>
     <row r="19">

</xml_diff>